<commit_message>
Free Trial Tracker: add "Next up" so a replacement is lined up before a trial ends
Both the web tracker on /bonus/ and the downloadable spreadsheet get a
"Next up (what replaces it)" field, a flag when a trial ends within 7 days
with nothing lined up (typing "none" dismisses it), and a summary count.
Entries saved before this change still load. Nothing is sent anywhere: the
web tracker still stores entries only in the visitor's browser.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TEeqpQpgSABNoFNcm8xK1o
</commit_message>
<xml_diff>
--- a/bonus/Subastian-Free-Trial-Tracker.xlsx
+++ b/bonus/Subastian-Free-Trial-Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Trial Tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trial Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -167,7 +167,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <font>
         <b val="1"/>
@@ -197,6 +197,18 @@
         <patternFill patternType="solid">
           <fgColor rgb="00DDF5E6"/>
           <bgColor rgb="00DDF5E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="FF9A5B00"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF1D6"/>
+          <bgColor rgb="FFFFF1D6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -562,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -575,6 +587,8 @@
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -624,6 +638,17 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Ending in 7 days with no next tool lined up</t>
+        </is>
+      </c>
+      <c r="D7" s="4">
+        <f>COUNTIF(L9:L38,"Line one up")</f>
+        <v/>
+      </c>
+    </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
@@ -675,6 +700,16 @@
           <t>Notes (cancel link, login email)</t>
         </is>
       </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>Next up (what replaces it)</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>Replacement check</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -718,6 +753,11 @@
           <t>Example row. Replace with your own.</t>
         </is>
       </c>
+      <c r="K9" s="12" t="n"/>
+      <c r="L9" s="9">
+        <f>IF(OR(I9&lt;&gt;"Active trial",F9=""),"",IF(LOWER(TRIM(K9))="none","Not needed",IF(K9&lt;&gt;"","Lined up",IF(AND(F9&gt;=0,F9&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -761,6 +801,11 @@
           <t>Example row. Replace with your own.</t>
         </is>
       </c>
+      <c r="K10" s="12" t="n"/>
+      <c r="L10" s="9">
+        <f>IF(OR(I10&lt;&gt;"Active trial",F10=""),"",IF(LOWER(TRIM(K10))="none","Not needed",IF(K10&lt;&gt;"","Lined up",IF(AND(F10&gt;=0,F10&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -803,6 +848,11 @@
         <is>
           <t>Example row. Replace with your own.</t>
         </is>
+      </c>
+      <c r="K11" s="12" t="n"/>
+      <c r="L11" s="9">
+        <f>IF(OR(I11&lt;&gt;"Active trial",F11=""),"",IF(LOWER(TRIM(K11))="none","Not needed",IF(K11&lt;&gt;"","Lined up",IF(AND(F11&gt;=0,F11&lt;=7),"Line one up",""))))</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -825,6 +875,11 @@
       </c>
       <c r="I12" s="7" t="n"/>
       <c r="J12" s="12" t="n"/>
+      <c r="K12" s="12" t="n"/>
+      <c r="L12" s="9">
+        <f>IF(OR(I12&lt;&gt;"Active trial",F12=""),"",IF(LOWER(TRIM(K12))="none","Not needed",IF(K12&lt;&gt;"","Lined up",IF(AND(F12&gt;=0,F12&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
@@ -846,6 +901,11 @@
       </c>
       <c r="I13" s="7" t="n"/>
       <c r="J13" s="12" t="n"/>
+      <c r="K13" s="12" t="n"/>
+      <c r="L13" s="9">
+        <f>IF(OR(I13&lt;&gt;"Active trial",F13=""),"",IF(LOWER(TRIM(K13))="none","Not needed",IF(K13&lt;&gt;"","Lined up",IF(AND(F13&gt;=0,F13&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -867,6 +927,11 @@
       </c>
       <c r="I14" s="7" t="n"/>
       <c r="J14" s="12" t="n"/>
+      <c r="K14" s="12" t="n"/>
+      <c r="L14" s="9">
+        <f>IF(OR(I14&lt;&gt;"Active trial",F14=""),"",IF(LOWER(TRIM(K14))="none","Not needed",IF(K14&lt;&gt;"","Lined up",IF(AND(F14&gt;=0,F14&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -888,6 +953,11 @@
       </c>
       <c r="I15" s="7" t="n"/>
       <c r="J15" s="12" t="n"/>
+      <c r="K15" s="12" t="n"/>
+      <c r="L15" s="9">
+        <f>IF(OR(I15&lt;&gt;"Active trial",F15=""),"",IF(LOWER(TRIM(K15))="none","Not needed",IF(K15&lt;&gt;"","Lined up",IF(AND(F15&gt;=0,F15&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
@@ -909,6 +979,11 @@
       </c>
       <c r="I16" s="7" t="n"/>
       <c r="J16" s="12" t="n"/>
+      <c r="K16" s="12" t="n"/>
+      <c r="L16" s="9">
+        <f>IF(OR(I16&lt;&gt;"Active trial",F16=""),"",IF(LOWER(TRIM(K16))="none","Not needed",IF(K16&lt;&gt;"","Lined up",IF(AND(F16&gt;=0,F16&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
@@ -930,6 +1005,11 @@
       </c>
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="12" t="n"/>
+      <c r="K17" s="12" t="n"/>
+      <c r="L17" s="9">
+        <f>IF(OR(I17&lt;&gt;"Active trial",F17=""),"",IF(LOWER(TRIM(K17))="none","Not needed",IF(K17&lt;&gt;"","Lined up",IF(AND(F17&gt;=0,F17&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
@@ -951,6 +1031,11 @@
       </c>
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="12" t="n"/>
+      <c r="K18" s="12" t="n"/>
+      <c r="L18" s="9">
+        <f>IF(OR(I18&lt;&gt;"Active trial",F18=""),"",IF(LOWER(TRIM(K18))="none","Not needed",IF(K18&lt;&gt;"","Lined up",IF(AND(F18&gt;=0,F18&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n"/>
@@ -972,6 +1057,11 @@
       </c>
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="12" t="n"/>
+      <c r="K19" s="12" t="n"/>
+      <c r="L19" s="9">
+        <f>IF(OR(I19&lt;&gt;"Active trial",F19=""),"",IF(LOWER(TRIM(K19))="none","Not needed",IF(K19&lt;&gt;"","Lined up",IF(AND(F19&gt;=0,F19&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n"/>
@@ -993,6 +1083,11 @@
       </c>
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="12" t="n"/>
+      <c r="K20" s="12" t="n"/>
+      <c r="L20" s="9">
+        <f>IF(OR(I20&lt;&gt;"Active trial",F20=""),"",IF(LOWER(TRIM(K20))="none","Not needed",IF(K20&lt;&gt;"","Lined up",IF(AND(F20&gt;=0,F20&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n"/>
@@ -1014,6 +1109,11 @@
       </c>
       <c r="I21" s="7" t="n"/>
       <c r="J21" s="12" t="n"/>
+      <c r="K21" s="12" t="n"/>
+      <c r="L21" s="9">
+        <f>IF(OR(I21&lt;&gt;"Active trial",F21=""),"",IF(LOWER(TRIM(K21))="none","Not needed",IF(K21&lt;&gt;"","Lined up",IF(AND(F21&gt;=0,F21&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n"/>
@@ -1035,6 +1135,11 @@
       </c>
       <c r="I22" s="7" t="n"/>
       <c r="J22" s="12" t="n"/>
+      <c r="K22" s="12" t="n"/>
+      <c r="L22" s="9">
+        <f>IF(OR(I22&lt;&gt;"Active trial",F22=""),"",IF(LOWER(TRIM(K22))="none","Not needed",IF(K22&lt;&gt;"","Lined up",IF(AND(F22&gt;=0,F22&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -1056,6 +1161,11 @@
       </c>
       <c r="I23" s="7" t="n"/>
       <c r="J23" s="12" t="n"/>
+      <c r="K23" s="12" t="n"/>
+      <c r="L23" s="9">
+        <f>IF(OR(I23&lt;&gt;"Active trial",F23=""),"",IF(LOWER(TRIM(K23))="none","Not needed",IF(K23&lt;&gt;"","Lined up",IF(AND(F23&gt;=0,F23&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n"/>
@@ -1077,6 +1187,11 @@
       </c>
       <c r="I24" s="7" t="n"/>
       <c r="J24" s="12" t="n"/>
+      <c r="K24" s="12" t="n"/>
+      <c r="L24" s="9">
+        <f>IF(OR(I24&lt;&gt;"Active trial",F24=""),"",IF(LOWER(TRIM(K24))="none","Not needed",IF(K24&lt;&gt;"","Lined up",IF(AND(F24&gt;=0,F24&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -1098,6 +1213,11 @@
       </c>
       <c r="I25" s="7" t="n"/>
       <c r="J25" s="12" t="n"/>
+      <c r="K25" s="12" t="n"/>
+      <c r="L25" s="9">
+        <f>IF(OR(I25&lt;&gt;"Active trial",F25=""),"",IF(LOWER(TRIM(K25))="none","Not needed",IF(K25&lt;&gt;"","Lined up",IF(AND(F25&gt;=0,F25&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n"/>
@@ -1119,6 +1239,11 @@
       </c>
       <c r="I26" s="7" t="n"/>
       <c r="J26" s="12" t="n"/>
+      <c r="K26" s="12" t="n"/>
+      <c r="L26" s="9">
+        <f>IF(OR(I26&lt;&gt;"Active trial",F26=""),"",IF(LOWER(TRIM(K26))="none","Not needed",IF(K26&lt;&gt;"","Lined up",IF(AND(F26&gt;=0,F26&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n"/>
@@ -1140,6 +1265,11 @@
       </c>
       <c r="I27" s="7" t="n"/>
       <c r="J27" s="12" t="n"/>
+      <c r="K27" s="12" t="n"/>
+      <c r="L27" s="9">
+        <f>IF(OR(I27&lt;&gt;"Active trial",F27=""),"",IF(LOWER(TRIM(K27))="none","Not needed",IF(K27&lt;&gt;"","Lined up",IF(AND(F27&gt;=0,F27&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n"/>
@@ -1161,6 +1291,11 @@
       </c>
       <c r="I28" s="7" t="n"/>
       <c r="J28" s="12" t="n"/>
+      <c r="K28" s="12" t="n"/>
+      <c r="L28" s="9">
+        <f>IF(OR(I28&lt;&gt;"Active trial",F28=""),"",IF(LOWER(TRIM(K28))="none","Not needed",IF(K28&lt;&gt;"","Lined up",IF(AND(F28&gt;=0,F28&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n"/>
@@ -1182,6 +1317,11 @@
       </c>
       <c r="I29" s="7" t="n"/>
       <c r="J29" s="12" t="n"/>
+      <c r="K29" s="12" t="n"/>
+      <c r="L29" s="9">
+        <f>IF(OR(I29&lt;&gt;"Active trial",F29=""),"",IF(LOWER(TRIM(K29))="none","Not needed",IF(K29&lt;&gt;"","Lined up",IF(AND(F29&gt;=0,F29&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n"/>
@@ -1203,6 +1343,11 @@
       </c>
       <c r="I30" s="7" t="n"/>
       <c r="J30" s="12" t="n"/>
+      <c r="K30" s="12" t="n"/>
+      <c r="L30" s="9">
+        <f>IF(OR(I30&lt;&gt;"Active trial",F30=""),"",IF(LOWER(TRIM(K30))="none","Not needed",IF(K30&lt;&gt;"","Lined up",IF(AND(F30&gt;=0,F30&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n"/>
@@ -1224,6 +1369,11 @@
       </c>
       <c r="I31" s="7" t="n"/>
       <c r="J31" s="12" t="n"/>
+      <c r="K31" s="12" t="n"/>
+      <c r="L31" s="9">
+        <f>IF(OR(I31&lt;&gt;"Active trial",F31=""),"",IF(LOWER(TRIM(K31))="none","Not needed",IF(K31&lt;&gt;"","Lined up",IF(AND(F31&gt;=0,F31&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n"/>
@@ -1245,6 +1395,11 @@
       </c>
       <c r="I32" s="7" t="n"/>
       <c r="J32" s="12" t="n"/>
+      <c r="K32" s="12" t="n"/>
+      <c r="L32" s="9">
+        <f>IF(OR(I32&lt;&gt;"Active trial",F32=""),"",IF(LOWER(TRIM(K32))="none","Not needed",IF(K32&lt;&gt;"","Lined up",IF(AND(F32&gt;=0,F32&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n"/>
@@ -1266,6 +1421,11 @@
       </c>
       <c r="I33" s="7" t="n"/>
       <c r="J33" s="12" t="n"/>
+      <c r="K33" s="12" t="n"/>
+      <c r="L33" s="9">
+        <f>IF(OR(I33&lt;&gt;"Active trial",F33=""),"",IF(LOWER(TRIM(K33))="none","Not needed",IF(K33&lt;&gt;"","Lined up",IF(AND(F33&gt;=0,F33&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n"/>
@@ -1287,6 +1447,11 @@
       </c>
       <c r="I34" s="7" t="n"/>
       <c r="J34" s="12" t="n"/>
+      <c r="K34" s="12" t="n"/>
+      <c r="L34" s="9">
+        <f>IF(OR(I34&lt;&gt;"Active trial",F34=""),"",IF(LOWER(TRIM(K34))="none","Not needed",IF(K34&lt;&gt;"","Lined up",IF(AND(F34&gt;=0,F34&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n"/>
@@ -1308,6 +1473,11 @@
       </c>
       <c r="I35" s="7" t="n"/>
       <c r="J35" s="12" t="n"/>
+      <c r="K35" s="12" t="n"/>
+      <c r="L35" s="9">
+        <f>IF(OR(I35&lt;&gt;"Active trial",F35=""),"",IF(LOWER(TRIM(K35))="none","Not needed",IF(K35&lt;&gt;"","Lined up",IF(AND(F35&gt;=0,F35&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n"/>
@@ -1329,6 +1499,11 @@
       </c>
       <c r="I36" s="7" t="n"/>
       <c r="J36" s="12" t="n"/>
+      <c r="K36" s="12" t="n"/>
+      <c r="L36" s="9">
+        <f>IF(OR(I36&lt;&gt;"Active trial",F36=""),"",IF(LOWER(TRIM(K36))="none","Not needed",IF(K36&lt;&gt;"","Lined up",IF(AND(F36&gt;=0,F36&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -1350,6 +1525,11 @@
       </c>
       <c r="I37" s="7" t="n"/>
       <c r="J37" s="12" t="n"/>
+      <c r="K37" s="12" t="n"/>
+      <c r="L37" s="9">
+        <f>IF(OR(I37&lt;&gt;"Active trial",F37=""),"",IF(LOWER(TRIM(K37))="none","Not needed",IF(K37&lt;&gt;"","Lined up",IF(AND(F37&gt;=0,F37&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n"/>
@@ -1371,6 +1551,11 @@
       </c>
       <c r="I38" s="7" t="n"/>
       <c r="J38" s="12" t="n"/>
+      <c r="K38" s="12" t="n"/>
+      <c r="L38" s="9">
+        <f>IF(OR(I38&lt;&gt;"Active trial",F38=""),"",IF(LOWER(TRIM(K38))="none","Not needed",IF(K38&lt;&gt;"","Lined up",IF(AND(F38&gt;=0,F38&lt;=7),"Line one up",""))))</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
@@ -1415,6 +1600,11 @@
   <conditionalFormatting sqref="I9:I38">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"Cancelled"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L9:L38">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"Line one up"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -1484,7 +1674,11 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr"/>
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>6. Before a trial ends, type what will replace it in "Next up". The sheet flags any trial ending within 7 days that has nothing lined up. Type "none" if you don't need one.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="18" t="inlineStr">

</xml_diff>